<commit_message>
Update wildlife findings export and rules
</commit_message>
<xml_diff>
--- a/wls_program/wildlife_parsing_codex_lookup.xlsx
+++ b/wls_program/wildlife_parsing_codex_lookup.xlsx
@@ -1166,7 +1166,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Rabbit / Hare</t>
+          <t>Snowshoe Hare</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1178,7 +1178,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Rabbit / Hare</t>
+          <t>Snowshoe Hare</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1190,7 +1190,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Rabbit / Hare</t>
+          <t>Snowshoe Hare</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1202,7 +1202,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Rabbit / Hare</t>
+          <t>Snowshoe Hare</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3164,7 +3164,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Rabbit / Hare</t>
+          <t>Snowshoe Hare</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -3174,7 +3174,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Rabbit Tracks</t>
+          <t>Snowshoe Hare Tracks</t>
         </is>
       </c>
     </row>
@@ -3189,7 +3189,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Rabbit / Hare</t>
+          <t>Snowshoe Hare</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -3199,7 +3199,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Rabbit Tracks</t>
+          <t>Snowshoe Hare Tracks</t>
         </is>
       </c>
     </row>
@@ -3214,7 +3214,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Rabbit / Hare</t>
+          <t>Snowshoe Hare</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -3224,7 +3224,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Rabbit Trail</t>
+          <t>Snowshoe Hare Trail</t>
         </is>
       </c>
     </row>
@@ -3239,7 +3239,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Rabbit / Hare</t>
+          <t>Snowshoe Hare</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -3249,7 +3249,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Rabbit Trail</t>
+          <t>Snowshoe Hare Trail</t>
         </is>
       </c>
     </row>
@@ -3939,7 +3939,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Rabbit / Hare</t>
+          <t>Snowshoe Hare</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -3949,7 +3949,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Rabbit Scat / Droppings</t>
+          <t>Snowshoe Hare Scat</t>
         </is>
       </c>
     </row>
@@ -3964,7 +3964,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Rabbit / Hare</t>
+          <t>Snowshoe Hare</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -3974,7 +3974,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Rabbit Scat / Droppings</t>
+          <t>Snowshoe Hare Scat</t>
         </is>
       </c>
     </row>
@@ -3989,7 +3989,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Rabbit / Hare</t>
+          <t>Snowshoe Hare</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -3999,7 +3999,7 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Rabbit Trail</t>
+          <t>Snowshoe Hare Trail</t>
         </is>
       </c>
     </row>
@@ -4014,7 +4014,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Rabbit / Hare</t>
+          <t>Snowshoe Hare</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -4024,7 +4024,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Rabbit Trail</t>
+          <t>Snowshoe Hare Trail</t>
         </is>
       </c>
     </row>
@@ -4039,7 +4039,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Rabbit / Hare</t>
+          <t>Snowshoe Hare</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -4049,7 +4049,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Rabbit Scat / Droppings</t>
+          <t>Snowshoe Hare Scat</t>
         </is>
       </c>
     </row>
@@ -4064,7 +4064,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Rabbit / Hare</t>
+          <t>Snowshoe Hare</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -4074,7 +4074,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Rabbit Tracks</t>
+          <t>Snowshoe Hare Tracks</t>
         </is>
       </c>
     </row>
@@ -4084,12 +4084,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>rabbit tracks</t>
+          <t>Snowshoe Hare Tracks</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Rabbit / Hare</t>
+          <t>Snowshoe Hare</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -4099,7 +4099,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Rabbit Tracks</t>
+          <t>Snowshoe Hare Tracks</t>
         </is>
       </c>
     </row>
@@ -4109,12 +4109,12 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>rabbit trail</t>
+          <t>Snowshoe Hare Trail</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Rabbit / Hare</t>
+          <t>Snowshoe Hare</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -4124,7 +4124,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Rabbit Trail</t>
+          <t>Snowshoe Hare Trail</t>
         </is>
       </c>
     </row>
@@ -4139,7 +4139,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Rabbit / Hare</t>
+          <t>Snowshoe Hare</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -4149,7 +4149,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Rabbit Trail</t>
+          <t>Snowshoe Hare Trail</t>
         </is>
       </c>
     </row>
@@ -7414,7 +7414,7 @@
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>Rabbit / Hare</t>
+          <t>Snowshoe Hare</t>
         </is>
       </c>
       <c r="D237" t="inlineStr">
@@ -7439,7 +7439,7 @@
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>Rabbit / Hare</t>
+          <t>Snowshoe Hare</t>
         </is>
       </c>
       <c r="D238" t="inlineStr">
@@ -7464,7 +7464,7 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>Rabbit / Hare</t>
+          <t>Snowshoe Hare</t>
         </is>
       </c>
       <c r="D239" t="inlineStr">
@@ -8829,7 +8829,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Rabbit / Hare</t>
+          <t>Snowshoe Hare</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -8839,7 +8839,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Rabbit Scat / Droppings</t>
+          <t>Snowshoe Hare Scat</t>
         </is>
       </c>
       <c r="F13" t="inlineStr"/>
@@ -8855,7 +8855,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Rabbit / Hare</t>
+          <t>Snowshoe Hare</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -8865,7 +8865,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Rabbit Tracks</t>
+          <t>Snowshoe Hare Tracks</t>
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
@@ -8881,7 +8881,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Rabbit / Hare</t>
+          <t>Snowshoe Hare</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -8891,7 +8891,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Rabbit Trail</t>
+          <t>Snowshoe Hare Trail</t>
         </is>
       </c>
       <c r="F15" t="inlineStr"/>
@@ -9140,7 +9140,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>(?=.*\bwoodpecker\b)(?=.*\b(cavity)\b).*</t>
+          <t>(?=.*\bwoodpecker\b)(?=.*\bcavity\b)(?=.*\btree(s)?\b).*</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -10523,7 +10523,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Rabbit / Hare</t>
+          <t>Snowshoe Hare</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -10553,7 +10553,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Rabbit / Hare</t>
+          <t>Snowshoe Hare</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -10999,6 +10999,336 @@
       <c r="F92" t="inlineStr">
         <is>
           <t>Last-resort fallback for any trail/path mention</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>1</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>^\s*pileated woodpecker feeding cavity\s*$</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Pileated Woodpecker Feeding Cavity</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Preserve exact pileated woodpecker cavity text instead of mapping to a generic woodpecker rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>1</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>^\s*moose browsing activity\s*$</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Moose Browsing Activity</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Preserve exact moose browsing activity text instead of mapping it to the generic browse/feeding sign bucket.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>1</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>^\s*(?:\d+\s+)?pileated woodpecker feeding cavity\s*$</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>[Keep Original]</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Preserve exact pileated woodpecker cavity text, including numbered prefixes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>1</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>^\s*(?:\d+\s+)?moose browsing activity\s*$</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>[Keep Original]</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Preserve exact moose browsing activity text.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>1</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>^\s*(?:\d+\s+)?moose hair\s*$</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>[Keep Original]</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>Preserve exact moose hair text instead of mapping to Moose Hair / Fur.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>1</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>^\s*(?:\d+\s+)?(?:inactive|nactive) small mammal den\s*$</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>[Keep Original]</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Preserve exact inactive small mammal den text.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>1</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>^\s*(?:\d+\s+)?red squirrel midden\s*$</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>[Keep Original]</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>Preserve exact red squirrel midden text instead of mapping to a generic squirrel rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="n">
+        <v>1</v>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>^\s*(?:\d+\s+)?coyote tracks\s*$</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>[Keep Original]</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>Preserve exact coyote tracks text instead of remapping to a broader canid label.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>1</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>^\s*(?:\d+\s+)?inactive mammal den\s*$</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>[Keep Original]</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>Preserve exact inactive mammal den text instead of remapping to inactive / possible den.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>1</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>^\s*(?:\d+\s+)?red squirrel burrow\s*$</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>[Keep Original]</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>Preserve exact red squirrel burrow text instead of remapping to squirrel sighting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>1</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>^\s*(?:\d+\s+)?field mouse hole mouse visual\s*$</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Small Mammal (Unidentified)</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Sighting</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Small Rodent Sighting</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>Map exact field mouse hole mouse visual text to Small Rodent Sighting.</t>
         </is>
       </c>
     </row>

</xml_diff>